<commit_message>
Fix #NAME? errors: FORMULATEXT needs the _xlfn. prefix (post-2007 function) when written by openpyxl
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_excel_operations.xlsx
+++ b/textbook_examples/mod01_excel_operations.xlsx
@@ -507,7 +507,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Column B computes the answer. Column C shows the formula that produced it, using FORMULATEXT().</t>
+          <t>Column B computes the answer. Column C shows the formula that produced it, using _xlfn.FORMULATEXT().</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>FORMULATEXT(B6)</f>
+        <f>_xlfn.FORMULATEXT(B6)</f>
         <v/>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -575,7 +575,7 @@
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>FORMULATEXT(B7)</f>
+        <f>_xlfn.FORMULATEXT(B7)</f>
         <v/>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>FORMULATEXT(B8)</f>
+        <f>_xlfn.FORMULATEXT(B8)</f>
         <v/>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>FORMULATEXT(B9)</f>
+        <f>_xlfn.FORMULATEXT(B9)</f>
         <v/>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -635,7 +635,7 @@
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>FORMULATEXT(B10)</f>
+        <f>_xlfn.FORMULATEXT(B10)</f>
         <v/>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -674,7 +674,7 @@
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>FORMULATEXT(B15)</f>
+        <f>_xlfn.FORMULATEXT(B15)</f>
         <v/>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -694,7 +694,7 @@
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>FORMULATEXT(B16)</f>
+        <f>_xlfn.FORMULATEXT(B16)</f>
         <v/>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -714,7 +714,7 @@
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>FORMULATEXT(B17)</f>
+        <f>_xlfn.FORMULATEXT(B17)</f>
         <v/>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -745,7 +745,7 @@
         <v/>
       </c>
       <c r="C20" s="9">
-        <f>FORMULATEXT(B20)</f>
+        <f>_xlfn.FORMULATEXT(B20)</f>
         <v/>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -765,7 +765,7 @@
         <v/>
       </c>
       <c r="C21" s="9">
-        <f>FORMULATEXT(B21)</f>
+        <f>_xlfn.FORMULATEXT(B21)</f>
         <v/>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
         <v/>
       </c>
       <c r="C22" s="9">
-        <f>FORMULATEXT(B22)</f>
+        <f>_xlfn.FORMULATEXT(B22)</f>
         <v/>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -805,7 +805,7 @@
         <v/>
       </c>
       <c r="C23" s="9">
-        <f>FORMULATEXT(B23)</f>
+        <f>_xlfn.FORMULATEXT(B23)</f>
         <v/>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         <v/>
       </c>
       <c r="C24" s="9">
-        <f>FORMULATEXT(B24)</f>
+        <f>_xlfn.FORMULATEXT(B24)</f>
         <v/>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -845,7 +845,7 @@
         <v/>
       </c>
       <c r="C25" s="9">
-        <f>FORMULATEXT(B25)</f>
+        <f>_xlfn.FORMULATEXT(B25)</f>
         <v/>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -876,7 +876,7 @@
         <v/>
       </c>
       <c r="C28" s="9">
-        <f>FORMULATEXT(B28)</f>
+        <f>_xlfn.FORMULATEXT(B28)</f>
         <v/>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
         <v/>
       </c>
       <c r="C29" s="9">
-        <f>FORMULATEXT(B29)</f>
+        <f>_xlfn.FORMULATEXT(B29)</f>
         <v/>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1005,7 +1005,7 @@
         <v/>
       </c>
       <c r="C39" s="9">
-        <f>FORMULATEXT(B39)</f>
+        <f>_xlfn.FORMULATEXT(B39)</f>
         <v/>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1076,7 +1076,7 @@
         <v/>
       </c>
       <c r="C44" s="9">
-        <f>FORMULATEXT(B44)</f>
+        <f>_xlfn.FORMULATEXT(B44)</f>
         <v/>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1135,7 +1135,7 @@
         <v/>
       </c>
       <c r="C50" s="9">
-        <f>FORMULATEXT(B50)</f>
+        <f>_xlfn.FORMULATEXT(B50)</f>
         <v/>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1155,7 +1155,7 @@
         <v/>
       </c>
       <c r="C51" s="9">
-        <f>FORMULATEXT(B51)</f>
+        <f>_xlfn.FORMULATEXT(B51)</f>
         <v/>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1197,7 +1197,7 @@
         <v/>
       </c>
       <c r="C53" s="9">
-        <f>FORMULATEXT(B53)</f>
+        <f>_xlfn.FORMULATEXT(B53)</f>
         <v/>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1217,7 +1217,7 @@
         <v/>
       </c>
       <c r="C54" s="9">
-        <f>FORMULATEXT(B54)</f>
+        <f>_xlfn.FORMULATEXT(B54)</f>
         <v/>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1237,7 +1237,7 @@
         <v/>
       </c>
       <c r="C55" s="9">
-        <f>FORMULATEXT(B55)</f>
+        <f>_xlfn.FORMULATEXT(B55)</f>
         <v/>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1251,9 +1251,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A13:D13"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A47:D47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Introduce AVERAGE and COUNT before the conditional versions
Chapter 2 opens with COUNTIF, SUMIF and AVERAGEIF, but only SUM had been
taught. Adds a short subsection covering the plain versions on the same five
fields, with a note on why the plain average of the yield column (52.5) differs
from the acreage-weighted figure (52.0), and a forward pointer to the
conditional functions.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_excel_operations.xlsx
+++ b/textbook_examples/mod01_excel_operations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_5DD97D7B509B8EEDB9EDB1704F5ED87656CDCAB8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E18AB39-782D-7943-A191-4FEA92BDE2CB}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_5DD97D7B509B8EEDB9EDB1704F5ED87656CDCAB8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40CC6D3B-EB08-7345-807D-47D54D6B6D58}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,9 +38,6 @@
     <t>Operators and the Order of Operations</t>
   </si>
   <si>
-    <t>Column B computes the answer. Column C shows the formula that produced it, using _xlfn.FORMULATEXT().</t>
-  </si>
-  <si>
     <t>What it does</t>
   </si>
   <si>
@@ -114,6 +111,9 @@
   </si>
   <si>
     <t xml:space="preserve">The ^ sign means 'to the power of'. </t>
+  </si>
+  <si>
+    <t>Column B computes the answer. Column C shows the formula that produced it.</t>
   </si>
 </sst>
 </file>
@@ -536,27 +536,27 @@
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -564,7 +564,7 @@
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" s="8">
         <f>12+5</f>
@@ -578,7 +578,7 @@
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="8">
         <f>12-5</f>
@@ -592,7 +592,7 @@
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="8">
         <f>12*5</f>
@@ -606,7 +606,7 @@
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="8">
         <f>12/5</f>
@@ -620,7 +620,7 @@
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="8">
         <f>12^2</f>
@@ -631,13 +631,13 @@
         <v>=12^2</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -645,7 +645,7 @@
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -654,7 +654,7 @@
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="8">
         <f>2+3*4</f>
@@ -665,12 +665,12 @@
         <v>=2+3*4</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="8">
         <f>(2+3)*4</f>
@@ -681,12 +681,12 @@
         <v>=(2+3)*4</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="8">
         <f>2*3^2</f>
@@ -697,14 +697,14 @@
         <v>=2*3^2</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -712,7 +712,7 @@
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="8">
         <f>100/2*5</f>
@@ -723,12 +723,12 @@
         <v>=100/2*5</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" s="8">
         <f>100/(2*5)</f>
@@ -739,13 +739,13 @@
         <v>=100/(2*5)</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>

</xml_diff>

<commit_message>
Chapter 7: video walkthroughs for Power Query and R-package downloads
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_excel_operations.xlsx
+++ b/textbook_examples/mod01_excel_operations.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -15,8 +15,11 @@
   <sheets>
     <sheet name="Formulas" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -38,12 +41,18 @@
     <t>Operators and the Order of Operations</t>
   </si>
   <si>
+    <t>Column B computes the answer. Column C shows the formula that produced it.</t>
+  </si>
+  <si>
     <t>What it does</t>
   </si>
   <si>
     <t>Result</t>
   </si>
   <si>
+    <t>Formula in col B</t>
+  </si>
+  <si>
     <t>Note</t>
   </si>
   <si>
@@ -65,6 +74,9 @@
     <t>Exponent</t>
   </si>
   <si>
+    <t xml:space="preserve">The ^ sign means 'to the power of'. </t>
+  </si>
+  <si>
     <t>Order of operations (PEMDAS)</t>
   </si>
   <si>
@@ -105,22 +117,13 @@
   </si>
   <si>
     <t>Same three numbers, two very different answers. When in doubt, add parentheses — they never hurt.</t>
-  </si>
-  <si>
-    <t>Formula in col B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The ^ sign means 'to the power of'. </t>
-  </si>
-  <si>
-    <t>Column B computes the answer. Column C shows the formula that produced it.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -215,9 +218,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -521,50 +524,50 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="18" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18" customHeight="1"/>
+    <row r="4" spans="1:4" ht="18" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="18" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" s="8">
         <f>12+5</f>
@@ -576,9 +579,9 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="18" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B7" s="8">
         <f>12-5</f>
@@ -590,9 +593,9 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="18" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" s="8">
         <f>12*5</f>
@@ -604,9 +607,9 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="18" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B9" s="8">
         <f>12/5</f>
@@ -618,9 +621,9 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="18" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" s="8">
         <f>12^2</f>
@@ -631,30 +634,30 @@
         <v>=12^2</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="18" customHeight="1"/>
+    <row r="12" spans="1:4" ht="18" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
     </row>
-    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="18" customHeight="1">
       <c r="A13" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
     </row>
-    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="18" customHeight="1"/>
+    <row r="15" spans="1:4" ht="18" customHeight="1">
       <c r="A15" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B15" s="8">
         <f>2+3*4</f>
@@ -665,12 +668,12 @@
         <v>=2+3*4</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="18" customHeight="1">
       <c r="A16" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B16" s="8">
         <f>(2+3)*4</f>
@@ -681,12 +684,12 @@
         <v>=(2+3)*4</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="18" customHeight="1">
       <c r="A17" s="7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B17" s="8">
         <f>2*3^2</f>
@@ -697,22 +700,22 @@
         <v>=2*3^2</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="18" customHeight="1"/>
+    <row r="19" spans="1:4" ht="18" customHeight="1"/>
+    <row r="20" spans="1:4" ht="18" customHeight="1">
       <c r="A20" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
     </row>
-    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="18" customHeight="1">
       <c r="A21" s="7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B21" s="8">
         <f>100/2*5</f>
@@ -723,12 +726,12 @@
         <v>=100/2*5</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="18" customHeight="1">
       <c r="A22" s="7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B22" s="8">
         <f>100/(2*5)</f>
@@ -739,21 +742,21 @@
         <v>=100/(2*5)</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="18" customHeight="1"/>
+    <row r="24" spans="1:4" ht="18" customHeight="1">
       <c r="A24" s="12" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
     </row>
-    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:4" ht="18" customHeight="1"/>
+    <row r="26" spans="1:4" ht="18" customHeight="1"/>
+    <row r="27" spans="1:4" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A13:D13"/>

</xml_diff>